<commit_message>
Interpolated profile for lake 71 (including one fix on original datasheet).  Fixed buoyancy frequency calculation.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/SuRGE/Shared Documents/data/CIN/CH4_071_Willowcreek/dataSheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\SuRGE\SuRGE_Sharepoint\data\CIN\CH4_071_Willowcreek\dataSheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="282" documentId="8_{C5CD2E9A-AC55-4F52-A58C-8568A1DAE714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C971E05-7B7B-4C6F-B545-53C2D1394674}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9DB011-2E92-44AF-B19B-0DE6E717EA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1833" yWindow="1833" windowWidth="19200" windowHeight="10034" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1225,7 +1225,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1247,9 +1247,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1275,11 +1272,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1288,14 +1281,7 @@
     <xf numFmtId="49" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1380,9 +1366,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1420,7 +1406,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1526,7 +1512,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1668,7 +1654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1677,211 +1663,211 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BQ17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" style="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.64453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.3515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.88671875" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.87890625" customWidth="1"/>
+    <col min="6" max="6" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.52734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.87890625" customWidth="1"/>
+    <col min="18" max="18" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.64453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.87890625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.41015625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.64453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.87890625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.64453125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.44140625" customWidth="1"/>
-    <col min="30" max="30" width="6.109375" customWidth="1"/>
+    <col min="29" max="29" width="6.41015625" customWidth="1"/>
+    <col min="30" max="30" width="6.1171875" customWidth="1"/>
     <col min="31" max="31" width="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.64453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.87890625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.3515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.64453125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.3515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.64453125" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.41015625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.64453125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="14.87890625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.64453125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.3515625" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="8" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="6.44140625" customWidth="1"/>
-    <col min="49" max="49" width="5.6640625" customWidth="1"/>
-    <col min="50" max="50" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6.41015625" customWidth="1"/>
+    <col min="49" max="49" width="5.64453125" customWidth="1"/>
+    <col min="50" max="50" width="6.3515625" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="11" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11.64453125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="8.87890625" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="10" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="16.1171875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="17.1171875" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="18.3515625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="13.64453125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="14" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="63" max="65" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="15.1171875" bestFit="1" customWidth="1"/>
+    <col min="63" max="65" width="9.1171875" bestFit="1" customWidth="1"/>
+    <col min="66" max="67" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.41015625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.3515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A1" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="36" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="37" t="s">
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="39" t="s">
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="39"/>
-      <c r="AH1" s="39"/>
-      <c r="AI1" s="39"/>
-      <c r="AJ1" s="39"/>
-      <c r="AK1" s="39"/>
-      <c r="AL1" s="39"/>
-      <c r="AM1" s="39"/>
-      <c r="AN1" s="39"/>
-      <c r="AO1" s="39"/>
-      <c r="AP1" s="39"/>
-      <c r="AQ1" s="39"/>
-      <c r="AR1" s="39"/>
-      <c r="AS1" s="39"/>
-      <c r="AT1" s="39"/>
-      <c r="AU1" s="39"/>
-      <c r="AV1" s="39"/>
-      <c r="AW1" s="39"/>
-      <c r="AX1" s="39"/>
-      <c r="AY1" s="39"/>
-      <c r="AZ1" s="39"/>
-      <c r="BA1" s="39"/>
-      <c r="BB1" s="39"/>
-      <c r="BC1" s="39"/>
-      <c r="BD1" s="39"/>
-      <c r="BE1" s="39"/>
-      <c r="BF1" s="39"/>
-      <c r="BG1" s="39"/>
-      <c r="BH1" s="39"/>
-      <c r="BI1" s="39"/>
-      <c r="BJ1" s="39"/>
-      <c r="BK1" s="38" t="s">
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="33"/>
+      <c r="AH1" s="33"/>
+      <c r="AI1" s="33"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" s="38"/>
-      <c r="BM1" s="38"/>
-      <c r="BN1" s="34" t="s">
+      <c r="BL1" s="32"/>
+      <c r="BM1" s="32"/>
+      <c r="BN1" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" s="34"/>
-      <c r="BP1" s="34"/>
-      <c r="BQ1" s="34"/>
-    </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="BO1" s="28"/>
+      <c r="BP1" s="28"/>
+      <c r="BQ1" s="28"/>
+    </row>
+    <row r="2" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="14" t="s">
+      <c r="Q2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="R2" s="13" t="s">
         <v>167</v>
       </c>
       <c r="S2" s="4" t="s">
@@ -1962,22 +1948,22 @@
       <c r="AR2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AS2" s="18" t="s">
+      <c r="AS2" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AT2" s="18" t="s">
+      <c r="AT2" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AU2" s="18" t="s">
+      <c r="AU2" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AV2" s="18" t="s">
+      <c r="AV2" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="AW2" s="18" t="s">
+      <c r="AW2" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="AX2" s="18" t="s">
+      <c r="AX2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="AY2" s="7" t="s">
@@ -2016,30 +2002,30 @@
       <c r="BJ2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="BK2" s="10" t="s">
+      <c r="BK2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="BL2" s="10" t="s">
+      <c r="BL2" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="BM2" s="10" t="s">
+      <c r="BM2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="BN2" s="11" t="s">
+      <c r="BN2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="BO2" s="11" t="s">
+      <c r="BO2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="BP2" s="25" t="s">
+      <c r="BP2" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="BQ2" s="25" t="s">
+      <c r="BQ2" s="22" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -2054,16 +2040,16 @@
       <c r="E3">
         <v>112.439201</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G3" s="31">
+      <c r="G3" s="25">
         <v>0.37638888888888888</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I3" s="31">
+      <c r="I3" s="25">
         <v>0.42222222222222222</v>
       </c>
       <c r="J3">
@@ -2072,10 +2058,10 @@
       <c r="L3" t="s">
         <v>174</v>
       </c>
-      <c r="S3" s="30" t="s">
+      <c r="S3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T3" s="32">
+      <c r="T3" s="26">
         <v>0.82598379629629637</v>
       </c>
       <c r="U3">
@@ -2121,7 +2107,7 @@
         <v>7.2</v>
       </c>
       <c r="AU3">
-        <v>0.49299999999999999</v>
+        <v>493</v>
       </c>
       <c r="AV3">
         <v>8.58</v>
@@ -2138,15 +2124,15 @@
       <c r="BO3">
         <v>407.42</v>
       </c>
-      <c r="BP3" s="30">
+      <c r="BP3" s="24">
         <v>44417</v>
       </c>
-      <c r="BQ3" s="32">
+      <c r="BQ3" s="26">
         <v>0.90543981481481473</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -2161,16 +2147,16 @@
       <c r="E4">
         <v>112.43634900000001</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="25">
         <v>0.41319444444444442</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="H4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="25">
         <v>0.64583333333333337</v>
       </c>
       <c r="J4">
@@ -2182,10 +2168,10 @@
       <c r="M4" t="s">
         <v>210</v>
       </c>
-      <c r="S4" s="30" t="s">
+      <c r="S4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T4" s="32">
+      <c r="T4" s="26">
         <v>8.1851851851851856E-2</v>
       </c>
       <c r="U4">
@@ -2248,15 +2234,15 @@
       <c r="BO4">
         <v>409.18</v>
       </c>
-      <c r="BP4" s="30">
+      <c r="BP4" s="24">
         <v>44418</v>
       </c>
-      <c r="BQ4" s="32">
+      <c r="BQ4" s="26">
         <v>0.11388888888888889</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -2274,10 +2260,10 @@
       <c r="R5" t="s">
         <v>215</v>
       </c>
-      <c r="S5" s="30" t="s">
+      <c r="S5" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="T5" s="33">
+      <c r="T5" s="27">
         <v>1.2100578703703704</v>
       </c>
       <c r="U5">
@@ -2344,8 +2330,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -2360,16 +2346,16 @@
       <c r="E6">
         <v>112.447816</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="25">
         <v>0.48749999999999999</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="25">
         <v>0.51666666666666672</v>
       </c>
       <c r="J6">
@@ -2384,10 +2370,10 @@
       <c r="P6" t="s">
         <v>178</v>
       </c>
-      <c r="S6" s="30" t="s">
+      <c r="S6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="26">
         <v>0.93321759259259263</v>
       </c>
       <c r="U6">
@@ -2445,8 +2431,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -2461,16 +2447,16 @@
       <c r="E7">
         <v>112.450141</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="25">
         <v>0.50347222222222221</v>
       </c>
-      <c r="H7" s="30" t="s">
+      <c r="H7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="25">
         <v>0.52777777777777779</v>
       </c>
       <c r="J7">
@@ -2485,10 +2471,10 @@
       <c r="P7" t="s">
         <v>181</v>
       </c>
-      <c r="S7" s="30" t="s">
+      <c r="S7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T7" s="32">
+      <c r="T7" s="26">
         <v>0.92736111111111119</v>
       </c>
       <c r="U7">
@@ -2546,8 +2532,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -2565,10 +2551,10 @@
       <c r="R8" t="s">
         <v>216</v>
       </c>
-      <c r="S8" s="30" t="s">
+      <c r="S8" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T8" s="32">
+      <c r="T8" s="26">
         <v>0.94166666666666676</v>
       </c>
       <c r="U8">
@@ -2626,8 +2612,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A9" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B9" t="s">
@@ -2645,10 +2631,10 @@
       <c r="R9" t="s">
         <v>216</v>
       </c>
-      <c r="S9" s="30" t="s">
+      <c r="S9" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T9" s="32">
+      <c r="T9" s="26">
         <v>0.95173611111111101</v>
       </c>
       <c r="U9">
@@ -2706,8 +2692,8 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A10" s="24" t="s">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A10" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B10" t="s">
@@ -2722,16 +2708,16 @@
       <c r="E10">
         <v>112.44584399999999</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="25">
         <v>0.53472222222222221</v>
       </c>
-      <c r="H10" s="30" t="s">
+      <c r="H10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="25">
         <v>0.5541666666666667</v>
       </c>
       <c r="J10">
@@ -2740,10 +2726,10 @@
       <c r="L10" t="s">
         <v>182</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="S10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T10" s="32">
+      <c r="T10" s="26">
         <v>0.96045138888888892</v>
       </c>
       <c r="U10">
@@ -2801,8 +2787,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A11" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B11" t="s">
@@ -2817,16 +2803,16 @@
       <c r="E11">
         <v>112.441974</v>
       </c>
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G11" s="31">
+      <c r="G11" s="25">
         <v>0.54583333333333328</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="H11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="25">
         <v>0.56597222222222221</v>
       </c>
       <c r="J11">
@@ -2841,10 +2827,10 @@
       <c r="P11" t="s">
         <v>185</v>
       </c>
-      <c r="S11" s="30" t="s">
+      <c r="S11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T11" s="32">
+      <c r="T11" s="26">
         <v>0.97037037037037033</v>
       </c>
       <c r="U11">
@@ -2902,8 +2888,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A12" s="24" t="s">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A12" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B12" t="s">
@@ -2918,14 +2904,14 @@
       <c r="E12">
         <v>112.445359</v>
       </c>
-      <c r="F12" s="30"/>
+      <c r="F12" s="24"/>
       <c r="R12" t="s">
         <v>216</v>
       </c>
-      <c r="S12" s="30" t="s">
+      <c r="S12" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T12" s="32">
+      <c r="T12" s="26">
         <v>2.1006944444444443E-2</v>
       </c>
       <c r="U12">
@@ -2983,8 +2969,8 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
+    <row r="13" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A13" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B13" t="s">
@@ -2999,25 +2985,25 @@
       <c r="E13">
         <v>112.44264699999999</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="25">
         <v>0.56388888888888888</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="25">
         <v>0.57500000000000007</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
-      <c r="S13" s="30" t="s">
+      <c r="S13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T13" s="32">
+      <c r="T13" s="26">
         <v>0.97891203703703711</v>
       </c>
       <c r="U13">
@@ -3075,8 +3061,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
+    <row r="14" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A14" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B14" t="s">
@@ -3094,10 +3080,10 @@
       <c r="R14" t="s">
         <v>217</v>
       </c>
-      <c r="S14" s="30" t="s">
+      <c r="S14" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T14" s="32">
+      <c r="T14" s="26">
         <v>5.6134259259259271E-3</v>
       </c>
       <c r="U14">
@@ -3155,8 +3141,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A15" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B15" t="s">
@@ -3171,14 +3157,14 @@
       <c r="E15">
         <v>112.43522900000001</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="24"/>
       <c r="R15" t="s">
         <v>218</v>
       </c>
-      <c r="S15" s="30" t="s">
+      <c r="S15" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T15" s="32">
+      <c r="T15" s="26">
         <v>7.7314814814814822E-2</v>
       </c>
       <c r="U15">
@@ -3236,8 +3222,8 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A16" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B16" t="s">
@@ -3252,16 +3238,16 @@
       <c r="E16">
         <v>112.432439</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="25">
         <v>0.50138888888888888</v>
       </c>
-      <c r="H16" s="30" t="s">
+      <c r="H16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="25">
         <v>0.63194444444444442</v>
       </c>
       <c r="J16">
@@ -3270,10 +3256,10 @@
       <c r="K16" t="s">
         <v>211</v>
       </c>
-      <c r="S16" s="30" t="s">
+      <c r="S16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T16" s="32">
+      <c r="T16" s="26">
         <v>4.0972222222222222E-2</v>
       </c>
       <c r="U16">
@@ -3331,8 +3317,8 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+    <row r="17" spans="1:50" x14ac:dyDescent="0.5">
+      <c r="A17" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B17" t="s">
@@ -3347,16 +3333,16 @@
       <c r="E17">
         <v>112.4300246</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="25">
         <v>0.5083333333333333</v>
       </c>
-      <c r="H17" s="30" t="s">
+      <c r="H17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="25">
         <v>0.65625</v>
       </c>
       <c r="J17">
@@ -3365,10 +3351,10 @@
       <c r="K17" t="s">
         <v>211</v>
       </c>
-      <c r="S17" s="30" t="s">
+      <c r="S17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T17" s="32">
+      <c r="T17" s="26">
         <v>6.340277777777778E-2</v>
       </c>
       <c r="U17">
@@ -3444,727 +3430,726 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{229CFC7D-096F-4A49-B44F-3C66E059D51A}">
   <dimension ref="A1:C73"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.1171875" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" style="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="116.6640625" style="26" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="26"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.64453125" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A1" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:3" ht="71.7" x14ac:dyDescent="0.5">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="23" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="26" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A15" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="26" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A19" t="s">
         <v>166</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" t="s">
         <v>170</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="C19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A20" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A21" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="26" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" t="s">
         <v>138</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="26" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A24" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="26" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A25" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="26" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A26" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" t="s">
         <v>170</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A27" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A28" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="26" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A29" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="B29" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="C29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="26" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A31" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="26" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A32" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="26" t="s">
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="26" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A33" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="B33" t="s">
         <v>96</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="26" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A34" t="s">
         <v>148</v>
       </c>
-      <c r="B34" s="26" t="s">
+      <c r="B34" t="s">
         <v>97</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="26" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" t="s">
         <v>99</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="26" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A36" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="26" t="s">
+      <c r="B36" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="26" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="26" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="26" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="26" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="26" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="26" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="26" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="26" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A44" t="s">
         <v>140</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="B44" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="26" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A45" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="26" t="s">
+      <c r="B45" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="26" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A46" t="s">
         <v>150</v>
       </c>
-      <c r="B46" s="26" t="s">
+      <c r="B46" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A47" t="s">
         <v>142</v>
       </c>
-      <c r="B47" s="26" t="s">
+      <c r="B47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A48" t="s">
         <v>29</v>
       </c>
-      <c r="B48" s="26" t="s">
+      <c r="B48" t="s">
         <v>119</v>
       </c>
-      <c r="C48" s="26" t="s">
+      <c r="C48" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="26" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A49" t="s">
         <v>30</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B49" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="26" t="s">
+      <c r="C49" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="26" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
         <v>31</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B50" t="s">
         <v>108</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C50" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="26" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A51" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="26" t="s">
+      <c r="B51" t="s">
         <v>109</v>
       </c>
-      <c r="C51" s="26" t="s">
+      <c r="C51" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="26" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A52" t="s">
         <v>33</v>
       </c>
-      <c r="B52" s="26" t="s">
+      <c r="B52" t="s">
         <v>110</v>
       </c>
-      <c r="C52" s="26" t="s">
+      <c r="C52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="26" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
         <v>151</v>
       </c>
-      <c r="B53" s="26" t="s">
+      <c r="B53" t="s">
         <v>111</v>
       </c>
-      <c r="C53" s="26" t="s">
+      <c r="C53" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="26" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="26" t="s">
+      <c r="B54" t="s">
         <v>112</v>
       </c>
-      <c r="C54" s="26" t="s">
+      <c r="C54" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="26" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
         <v>40</v>
       </c>
-      <c r="B55" s="26" t="s">
+      <c r="B55" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="26" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A56" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="26" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="26" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="26" t="s">
+      <c r="B58" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="26" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
         <v>152</v>
       </c>
-      <c r="B59" s="26" t="s">
+      <c r="B59" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="26" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="26" t="s">
+      <c r="B60" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="26" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="26" t="s">
+      <c r="B61" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="26" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
         <v>144</v>
       </c>
-      <c r="B62" s="26" t="s">
+      <c r="B62" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="26" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
         <v>145</v>
       </c>
-      <c r="B63" s="26" t="s">
+      <c r="B63" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="26" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A64" t="s">
         <v>146</v>
       </c>
-      <c r="B64" s="26" t="s">
+      <c r="B64" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="26" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A65" t="s">
         <v>153</v>
       </c>
-      <c r="B65" s="26" t="s">
+      <c r="B65" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="26" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A66" t="s">
         <v>147</v>
       </c>
-      <c r="B66" s="26" t="s">
+      <c r="B66" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="26" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A67" t="s">
         <v>49</v>
       </c>
-      <c r="B67" s="26" t="s">
+      <c r="B67" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="26" t="s">
+      <c r="C67" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="26" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A68" t="s">
         <v>50</v>
       </c>
-      <c r="B68" s="26" t="s">
+      <c r="B68" t="s">
         <v>121</v>
       </c>
-      <c r="C68" s="26" t="s">
+      <c r="C68" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="26" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A69" t="s">
         <v>51</v>
       </c>
-      <c r="B69" s="26" t="s">
+      <c r="B69" t="s">
         <v>122</v>
       </c>
-      <c r="C69" s="26" t="s">
+      <c r="C69" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="26" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A70" t="s">
         <v>52</v>
       </c>
-      <c r="B70" s="26" t="s">
+      <c r="B70" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="26" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A71" t="s">
         <v>53</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" t="s">
         <v>161</v>
       </c>
-      <c r="C71" s="26" t="s">
+      <c r="C71" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="26" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A72" t="s">
         <v>162</v>
       </c>
-      <c r="B72" s="26" t="s">
+      <c r="B72" t="s">
         <v>163</v>
       </c>
-      <c r="C72" s="26" t="s">
+      <c r="C72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="26" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A73" t="s">
         <v>164</v>
       </c>
-      <c r="B73" s="26" t="s">
+      <c r="B73" t="s">
         <v>165</v>
       </c>
-      <c r="C73" s="26" t="s">
+      <c r="C73" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4176,33 +4161,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081A6BD0-DB1A-406D-A526-8D337C57DAFE}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="24"/>
-    <col min="3" max="3" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8.87890625" style="21"/>
+    <col min="3" max="3" width="15.41015625" customWidth="1"/>
+    <col min="5" max="5" width="13.3515625" customWidth="1"/>
+    <col min="7" max="7" width="12.3515625" customWidth="1"/>
+    <col min="9" max="9" width="14.3515625" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A1" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4218,7 +4200,7 @@
       <c r="E2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -4236,8 +4218,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -4265,8 +4247,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -4294,8 +4276,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -4323,8 +4305,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -4352,8 +4334,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -4381,8 +4363,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -4422,14 +4404,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FA2781-11F0-42BE-92DB-835D44D19C85}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5546875" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.52734375" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -4440,7 +4422,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4451,7 +4433,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -4462,19 +4444,19 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A4" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B5" t="s">
@@ -4484,8 +4466,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
@@ -4495,16 +4477,16 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" s="18" t="s">
         <v>123</v>
       </c>
       <c r="B8" t="s">
@@ -4514,8 +4496,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" s="18" t="s">
         <v>124</v>
       </c>
       <c r="B9" t="s">
@@ -4525,8 +4507,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" s="19" t="s">
         <v>125</v>
       </c>
       <c r="B10" t="s">
@@ -4536,8 +4518,8 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" s="18" t="s">
         <v>158</v>
       </c>
       <c r="B11" t="s">
@@ -4595,6 +4577,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5065,20 +5061,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
@@ -5094,7 +5076,11 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5106,9 +5092,24 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="8b03727f-4454-4722-b3e6-018d8dcaf2fd"/>
+    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revert "Interpolated profile for lake 71... This should bring us back to Jake's Jan 9 2026 commit."
This reverts commit 3525eb6897a719d9642990d2767a5d28774d70ac.
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\SuRGE\SuRGE_Sharepoint\data\CIN\CH4_071_Willowcreek\dataSheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/SuRGE/Shared Documents/data/CIN/CH4_071_Willowcreek/dataSheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9DB011-2E92-44AF-B19B-0DE6E717EA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="282" documentId="8_{C5CD2E9A-AC55-4F52-A58C-8568A1DAE714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C971E05-7B7B-4C6F-B545-53C2D1394674}"/>
   <bookViews>
-    <workbookView xWindow="1833" yWindow="1833" windowWidth="19200" windowHeight="10034" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1225,7 +1225,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1247,6 +1247,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1272,7 +1275,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1281,7 +1288,14 @@
     <xf numFmtId="49" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1366,9 +1380,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1406,7 +1420,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1512,7 +1526,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1654,7 +1668,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1663,211 +1677,211 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BQ17"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.64453125" style="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.3515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.87890625" customWidth="1"/>
-    <col min="6" max="6" width="14.41015625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.52734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="13.3515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.52734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.41015625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.87890625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.41015625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.87890625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.41015625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.87890625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.87890625" customWidth="1"/>
-    <col min="18" max="18" width="15.41015625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.64453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.87890625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.64453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.41015625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.64453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.87890625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.41015625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.87890625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.64453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.88671875" customWidth="1"/>
+    <col min="18" max="18" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.41015625" customWidth="1"/>
-    <col min="30" max="30" width="6.1171875" customWidth="1"/>
+    <col min="29" max="29" width="6.44140625" customWidth="1"/>
+    <col min="30" max="30" width="6.109375" customWidth="1"/>
     <col min="31" max="31" width="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.64453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.52734375" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.87890625" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.3515625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.52734375" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.64453125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.3515625" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.64453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.41015625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13.64453125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.87890625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.64453125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.3515625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="8" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.3515625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="6.41015625" customWidth="1"/>
-    <col min="49" max="49" width="5.64453125" customWidth="1"/>
-    <col min="50" max="50" width="6.3515625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6.44140625" customWidth="1"/>
+    <col min="49" max="49" width="5.6640625" customWidth="1"/>
+    <col min="50" max="50" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="11" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="11.64453125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="13.3515625" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.52734375" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="8.87890625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="10" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="16.1171875" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="17.1171875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="18.3515625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.64453125" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="14" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="15.1171875" bestFit="1" customWidth="1"/>
-    <col min="63" max="65" width="9.1171875" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="9.3515625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="17.41015625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.3515625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="63" max="65" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="66" max="67" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A1" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="30" t="s">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="31" t="s">
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="33" t="s">
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="37"/>
+      <c r="X1" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="33"/>
-      <c r="Z1" s="33"/>
-      <c r="AA1" s="33"/>
-      <c r="AB1" s="33"/>
-      <c r="AC1" s="33"/>
-      <c r="AD1" s="33"/>
-      <c r="AE1" s="33"/>
-      <c r="AF1" s="33"/>
-      <c r="AG1" s="33"/>
-      <c r="AH1" s="33"/>
-      <c r="AI1" s="33"/>
-      <c r="AJ1" s="33"/>
-      <c r="AK1" s="33"/>
-      <c r="AL1" s="33"/>
-      <c r="AM1" s="33"/>
-      <c r="AN1" s="33"/>
-      <c r="AO1" s="33"/>
-      <c r="AP1" s="33"/>
-      <c r="AQ1" s="33"/>
-      <c r="AR1" s="33"/>
-      <c r="AS1" s="33"/>
-      <c r="AT1" s="33"/>
-      <c r="AU1" s="33"/>
-      <c r="AV1" s="33"/>
-      <c r="AW1" s="33"/>
-      <c r="AX1" s="33"/>
-      <c r="AY1" s="33"/>
-      <c r="AZ1" s="33"/>
-      <c r="BA1" s="33"/>
-      <c r="BB1" s="33"/>
-      <c r="BC1" s="33"/>
-      <c r="BD1" s="33"/>
-      <c r="BE1" s="33"/>
-      <c r="BF1" s="33"/>
-      <c r="BG1" s="33"/>
-      <c r="BH1" s="33"/>
-      <c r="BI1" s="33"/>
-      <c r="BJ1" s="33"/>
-      <c r="BK1" s="32" t="s">
+      <c r="Y1" s="39"/>
+      <c r="Z1" s="39"/>
+      <c r="AA1" s="39"/>
+      <c r="AB1" s="39"/>
+      <c r="AC1" s="39"/>
+      <c r="AD1" s="39"/>
+      <c r="AE1" s="39"/>
+      <c r="AF1" s="39"/>
+      <c r="AG1" s="39"/>
+      <c r="AH1" s="39"/>
+      <c r="AI1" s="39"/>
+      <c r="AJ1" s="39"/>
+      <c r="AK1" s="39"/>
+      <c r="AL1" s="39"/>
+      <c r="AM1" s="39"/>
+      <c r="AN1" s="39"/>
+      <c r="AO1" s="39"/>
+      <c r="AP1" s="39"/>
+      <c r="AQ1" s="39"/>
+      <c r="AR1" s="39"/>
+      <c r="AS1" s="39"/>
+      <c r="AT1" s="39"/>
+      <c r="AU1" s="39"/>
+      <c r="AV1" s="39"/>
+      <c r="AW1" s="39"/>
+      <c r="AX1" s="39"/>
+      <c r="AY1" s="39"/>
+      <c r="AZ1" s="39"/>
+      <c r="BA1" s="39"/>
+      <c r="BB1" s="39"/>
+      <c r="BC1" s="39"/>
+      <c r="BD1" s="39"/>
+      <c r="BE1" s="39"/>
+      <c r="BF1" s="39"/>
+      <c r="BG1" s="39"/>
+      <c r="BH1" s="39"/>
+      <c r="BI1" s="39"/>
+      <c r="BJ1" s="39"/>
+      <c r="BK1" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" s="32"/>
-      <c r="BM1" s="32"/>
-      <c r="BN1" s="28" t="s">
+      <c r="BL1" s="38"/>
+      <c r="BM1" s="38"/>
+      <c r="BN1" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" s="28"/>
-      <c r="BP1" s="28"/>
-      <c r="BQ1" s="28"/>
-    </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A2" s="20" t="s">
+      <c r="BO1" s="34"/>
+      <c r="BP1" s="34"/>
+      <c r="BQ1" s="34"/>
+    </row>
+    <row r="2" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="13" t="s">
+      <c r="R2" s="14" t="s">
         <v>167</v>
       </c>
       <c r="S2" s="4" t="s">
@@ -1948,22 +1962,22 @@
       <c r="AR2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AS2" s="17" t="s">
+      <c r="AS2" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="AT2" s="17" t="s">
+      <c r="AT2" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="AU2" s="17" t="s">
+      <c r="AU2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="AV2" s="17" t="s">
+      <c r="AV2" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="AW2" s="17" t="s">
+      <c r="AW2" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="AX2" s="17" t="s">
+      <c r="AX2" s="18" t="s">
         <v>34</v>
       </c>
       <c r="AY2" s="7" t="s">
@@ -2002,30 +2016,30 @@
       <c r="BJ2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="BK2" s="9" t="s">
+      <c r="BK2" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="BL2" s="9" t="s">
+      <c r="BL2" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="BM2" s="9" t="s">
+      <c r="BM2" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="BN2" s="10" t="s">
+      <c r="BN2" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="BO2" s="10" t="s">
+      <c r="BO2" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="BP2" s="22" t="s">
+      <c r="BP2" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="BQ2" s="22" t="s">
+      <c r="BQ2" s="25" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A3" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -2040,16 +2054,16 @@
       <c r="E3">
         <v>112.439201</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="31">
         <v>0.37638888888888888</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I3" s="25">
+      <c r="I3" s="31">
         <v>0.42222222222222222</v>
       </c>
       <c r="J3">
@@ -2058,10 +2072,10 @@
       <c r="L3" t="s">
         <v>174</v>
       </c>
-      <c r="S3" s="24" t="s">
+      <c r="S3" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T3" s="26">
+      <c r="T3" s="32">
         <v>0.82598379629629637</v>
       </c>
       <c r="U3">
@@ -2107,7 +2121,7 @@
         <v>7.2</v>
       </c>
       <c r="AU3">
-        <v>493</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="AV3">
         <v>8.58</v>
@@ -2124,15 +2138,15 @@
       <c r="BO3">
         <v>407.42</v>
       </c>
-      <c r="BP3" s="24">
+      <c r="BP3" s="30">
         <v>44417</v>
       </c>
-      <c r="BQ3" s="26">
+      <c r="BQ3" s="32">
         <v>0.90543981481481473</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -2147,16 +2161,16 @@
       <c r="E4">
         <v>112.43634900000001</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="31">
         <v>0.41319444444444442</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="H4" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="31">
         <v>0.64583333333333337</v>
       </c>
       <c r="J4">
@@ -2168,10 +2182,10 @@
       <c r="M4" t="s">
         <v>210</v>
       </c>
-      <c r="S4" s="24" t="s">
+      <c r="S4" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T4" s="26">
+      <c r="T4" s="32">
         <v>8.1851851851851856E-2</v>
       </c>
       <c r="U4">
@@ -2234,15 +2248,15 @@
       <c r="BO4">
         <v>409.18</v>
       </c>
-      <c r="BP4" s="24">
+      <c r="BP4" s="30">
         <v>44418</v>
       </c>
-      <c r="BQ4" s="26">
+      <c r="BQ4" s="32">
         <v>0.11388888888888889</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -2260,10 +2274,10 @@
       <c r="R5" t="s">
         <v>215</v>
       </c>
-      <c r="S5" s="24" t="s">
+      <c r="S5" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="T5" s="27">
+      <c r="T5" s="33">
         <v>1.2100578703703704</v>
       </c>
       <c r="U5">
@@ -2330,8 +2344,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -2346,16 +2360,16 @@
       <c r="E6">
         <v>112.447816</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G6" s="25">
+      <c r="G6" s="31">
         <v>0.48749999999999999</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="31">
         <v>0.51666666666666672</v>
       </c>
       <c r="J6">
@@ -2370,10 +2384,10 @@
       <c r="P6" t="s">
         <v>178</v>
       </c>
-      <c r="S6" s="24" t="s">
+      <c r="S6" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T6" s="26">
+      <c r="T6" s="32">
         <v>0.93321759259259263</v>
       </c>
       <c r="U6">
@@ -2431,8 +2445,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -2447,16 +2461,16 @@
       <c r="E7">
         <v>112.450141</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="F7" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="31">
         <v>0.50347222222222221</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I7" s="25">
+      <c r="I7" s="31">
         <v>0.52777777777777779</v>
       </c>
       <c r="J7">
@@ -2471,10 +2485,10 @@
       <c r="P7" t="s">
         <v>181</v>
       </c>
-      <c r="S7" s="24" t="s">
+      <c r="S7" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T7" s="26">
+      <c r="T7" s="32">
         <v>0.92736111111111119</v>
       </c>
       <c r="U7">
@@ -2532,8 +2546,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A8" s="21" t="s">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -2551,10 +2565,10 @@
       <c r="R8" t="s">
         <v>216</v>
       </c>
-      <c r="S8" s="24" t="s">
+      <c r="S8" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T8" s="26">
+      <c r="T8" s="32">
         <v>0.94166666666666676</v>
       </c>
       <c r="U8">
@@ -2612,8 +2626,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A9" s="21" t="s">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B9" t="s">
@@ -2631,10 +2645,10 @@
       <c r="R9" t="s">
         <v>216</v>
       </c>
-      <c r="S9" s="24" t="s">
+      <c r="S9" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T9" s="26">
+      <c r="T9" s="32">
         <v>0.95173611111111101</v>
       </c>
       <c r="U9">
@@ -2692,8 +2706,8 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A10" s="21" t="s">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A10" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B10" t="s">
@@ -2708,16 +2722,16 @@
       <c r="E10">
         <v>112.44584399999999</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G10" s="25">
+      <c r="G10" s="31">
         <v>0.53472222222222221</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="31">
         <v>0.5541666666666667</v>
       </c>
       <c r="J10">
@@ -2726,10 +2740,10 @@
       <c r="L10" t="s">
         <v>182</v>
       </c>
-      <c r="S10" s="24" t="s">
+      <c r="S10" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T10" s="26">
+      <c r="T10" s="32">
         <v>0.96045138888888892</v>
       </c>
       <c r="U10">
@@ -2787,8 +2801,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A11" s="21" t="s">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A11" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B11" t="s">
@@ -2803,16 +2817,16 @@
       <c r="E11">
         <v>112.441974</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="F11" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G11" s="25">
+      <c r="G11" s="31">
         <v>0.54583333333333328</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I11" s="25">
+      <c r="I11" s="31">
         <v>0.56597222222222221</v>
       </c>
       <c r="J11">
@@ -2827,10 +2841,10 @@
       <c r="P11" t="s">
         <v>185</v>
       </c>
-      <c r="S11" s="24" t="s">
+      <c r="S11" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T11" s="26">
+      <c r="T11" s="32">
         <v>0.97037037037037033</v>
       </c>
       <c r="U11">
@@ -2888,8 +2902,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A12" s="21" t="s">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A12" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B12" t="s">
@@ -2904,14 +2918,14 @@
       <c r="E12">
         <v>112.445359</v>
       </c>
-      <c r="F12" s="24"/>
+      <c r="F12" s="30"/>
       <c r="R12" t="s">
         <v>216</v>
       </c>
-      <c r="S12" s="24" t="s">
+      <c r="S12" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T12" s="26">
+      <c r="T12" s="32">
         <v>2.1006944444444443E-2</v>
       </c>
       <c r="U12">
@@ -2969,8 +2983,8 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A13" s="21" t="s">
+    <row r="13" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A13" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B13" t="s">
@@ -2985,25 +2999,25 @@
       <c r="E13">
         <v>112.44264699999999</v>
       </c>
-      <c r="F13" s="24" t="s">
+      <c r="F13" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="31">
         <v>0.56388888888888888</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I13" s="25">
+      <c r="I13" s="31">
         <v>0.57500000000000007</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
-      <c r="S13" s="24" t="s">
+      <c r="S13" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T13" s="26">
+      <c r="T13" s="32">
         <v>0.97891203703703711</v>
       </c>
       <c r="U13">
@@ -3061,8 +3075,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A14" s="21" t="s">
+    <row r="14" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B14" t="s">
@@ -3080,10 +3094,10 @@
       <c r="R14" t="s">
         <v>217</v>
       </c>
-      <c r="S14" s="24" t="s">
+      <c r="S14" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T14" s="26">
+      <c r="T14" s="32">
         <v>5.6134259259259271E-3</v>
       </c>
       <c r="U14">
@@ -3141,8 +3155,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A15" s="21" t="s">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A15" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B15" t="s">
@@ -3157,14 +3171,14 @@
       <c r="E15">
         <v>112.43522900000001</v>
       </c>
-      <c r="F15" s="24"/>
+      <c r="F15" s="30"/>
       <c r="R15" t="s">
         <v>218</v>
       </c>
-      <c r="S15" s="24" t="s">
+      <c r="S15" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T15" s="26">
+      <c r="T15" s="32">
         <v>7.7314814814814822E-2</v>
       </c>
       <c r="U15">
@@ -3222,8 +3236,8 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.5">
-      <c r="A16" s="21" t="s">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.3">
+      <c r="A16" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B16" t="s">
@@ -3238,16 +3252,16 @@
       <c r="E16">
         <v>112.432439</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="31">
         <v>0.50138888888888888</v>
       </c>
-      <c r="H16" s="24" t="s">
+      <c r="H16" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="31">
         <v>0.63194444444444442</v>
       </c>
       <c r="J16">
@@ -3256,10 +3270,10 @@
       <c r="K16" t="s">
         <v>211</v>
       </c>
-      <c r="S16" s="24" t="s">
+      <c r="S16" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T16" s="26">
+      <c r="T16" s="32">
         <v>4.0972222222222222E-2</v>
       </c>
       <c r="U16">
@@ -3317,8 +3331,8 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.5">
-      <c r="A17" s="21" t="s">
+    <row r="17" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B17" t="s">
@@ -3333,16 +3347,16 @@
       <c r="E17">
         <v>112.4300246</v>
       </c>
-      <c r="F17" s="24" t="s">
+      <c r="F17" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="25">
+      <c r="G17" s="31">
         <v>0.5083333333333333</v>
       </c>
-      <c r="H17" s="24" t="s">
+      <c r="H17" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="I17" s="25">
+      <c r="I17" s="31">
         <v>0.65625</v>
       </c>
       <c r="J17">
@@ -3351,10 +3365,10 @@
       <c r="K17" t="s">
         <v>211</v>
       </c>
-      <c r="S17" s="24" t="s">
+      <c r="S17" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="T17" s="26">
+      <c r="T17" s="32">
         <v>6.340277777777778E-2</v>
       </c>
       <c r="U17">
@@ -3430,726 +3444,727 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{229CFC7D-096F-4A49-B44F-3C66E059D51A}">
   <dimension ref="A1:C73"/>
-  <sheetFormatPr defaultColWidth="9.1171875" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="116.64453125" customWidth="1"/>
-    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" style="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.6640625" style="26" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" style="26" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.109375" style="26"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="26" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="26" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="26" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.7" x14ac:dyDescent="0.5">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="A4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="28" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="26" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A6" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="26" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A7" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="26" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="26" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A9" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="26" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A10" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="26" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A11" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="26" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A12" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="29" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A13" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A14" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="26" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A15" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A16" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="26" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A17" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A18" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="26" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A19" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A20" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="26" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A21" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="26" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A22" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="26" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A23" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="26" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A24" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A25" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A26" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="26" t="s">
         <v>170</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A27" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="26" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A28" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="26" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A29" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="26" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A30" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="26" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A31" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="26" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A32" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="26" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A33" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A34" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="26" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A35" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="26" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A36" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="26" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A37" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="26" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A38" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="26" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A39" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="26" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A40" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="26" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A41" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="26" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A42" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A43" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A44" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A45" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A46" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A47" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A48" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="26" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A49" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="26" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A50" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="26" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A51" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="26" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A52" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A53" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="26" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A54" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C54" s="26" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A55" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="26" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A56" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="26" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A57" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="26" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A58" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="26" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A59" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="26" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A60" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="26" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A61" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A62" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A63" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A64" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A65" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A66" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="26" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A67" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A68" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C68" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A69" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C69" s="26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A70" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C70" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A71" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="26" t="s">
         <v>161</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C71" s="26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A72" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C72" s="26" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A73" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C73" s="26" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4161,30 +4176,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081A6BD0-DB1A-406D-A526-8D337C57DAFE}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.87890625" style="21"/>
-    <col min="3" max="3" width="15.41015625" customWidth="1"/>
-    <col min="5" max="5" width="13.3515625" customWidth="1"/>
-    <col min="7" max="7" width="12.3515625" customWidth="1"/>
-    <col min="9" max="9" width="14.3515625" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="24"/>
+    <col min="3" max="3" width="15.44140625" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4200,7 +4218,7 @@
       <c r="E2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="9" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -4218,8 +4236,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A3" s="21" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -4247,8 +4265,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -4276,8 +4294,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -4305,8 +4323,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -4334,8 +4352,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -4363,8 +4381,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A8" s="21" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -4404,14 +4422,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FA2781-11F0-42BE-92DB-835D44D19C85}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.52734375" customWidth="1"/>
-    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.5546875" customWidth="1"/>
+    <col min="3" max="3" width="49.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -4422,7 +4440,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4433,7 +4451,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -4444,19 +4462,19 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A4" s="18" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="17" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A5" s="18" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
         <v>46</v>
       </c>
       <c r="B5" t="s">
@@ -4466,8 +4484,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A6" s="18" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
@@ -4477,16 +4495,16 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A7" s="18" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
         <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A8" s="18" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>123</v>
       </c>
       <c r="B8" t="s">
@@ -4496,8 +4514,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A9" s="18" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>124</v>
       </c>
       <c r="B9" t="s">
@@ -4507,8 +4525,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A10" s="19" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
         <v>125</v>
       </c>
       <c r="B10" t="s">
@@ -4518,8 +4536,8 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
-      <c r="A11" s="18" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
         <v>158</v>
       </c>
       <c r="B11" t="s">
@@ -4577,20 +4595,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5061,6 +5065,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
@@ -5076,11 +5094,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5092,24 +5106,9 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="8b03727f-4454-4722-b3e6-018d8dcaf2fd"/>
-    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changed buoyancy frequency calculation, added profile from lake 71, edited conductivity value for lake 71, updated files 5, 6, and 7
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/SuRGE/Shared Documents/data/CIN/CH4_071_Willowcreek/dataSheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\SuRGE\SuRGE_Sharepoint\data\CIN\CH4_071_Willowcreek\dataSheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="282" documentId="8_{C5CD2E9A-AC55-4F52-A58C-8568A1DAE714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C971E05-7B7B-4C6F-B545-53C2D1394674}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD1EDDA7-7E6B-49BC-BA47-29BA968DB3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1225,7 +1225,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1247,9 +1247,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1275,11 +1272,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1288,14 +1281,7 @@
     <xf numFmtId="49" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1380,9 +1366,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1420,7 +1406,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1526,7 +1512,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1668,7 +1654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1677,211 +1663,211 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BQ17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" style="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.64453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.3515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.88671875" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.87890625" customWidth="1"/>
+    <col min="6" max="6" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.52734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.87890625" customWidth="1"/>
+    <col min="18" max="18" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.64453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.87890625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.41015625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.64453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.87890625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.64453125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.44140625" customWidth="1"/>
-    <col min="30" max="30" width="6.109375" customWidth="1"/>
+    <col min="29" max="29" width="6.41015625" customWidth="1"/>
+    <col min="30" max="30" width="6.1171875" customWidth="1"/>
     <col min="31" max="31" width="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.64453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.87890625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.3515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.64453125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.3515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.64453125" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.41015625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.64453125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="14.87890625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.64453125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.3515625" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="8" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="6.44140625" customWidth="1"/>
-    <col min="49" max="49" width="5.6640625" customWidth="1"/>
-    <col min="50" max="50" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6.41015625" customWidth="1"/>
+    <col min="49" max="49" width="5.64453125" customWidth="1"/>
+    <col min="50" max="50" width="6.3515625" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="11" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11.64453125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="8.87890625" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="10" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="16.1171875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="17.1171875" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="18.3515625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="13.64453125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="14" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="63" max="65" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="15.1171875" bestFit="1" customWidth="1"/>
+    <col min="63" max="65" width="9.1171875" bestFit="1" customWidth="1"/>
+    <col min="66" max="67" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.41015625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.3515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A1" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="36" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="37" t="s">
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="39" t="s">
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="39"/>
-      <c r="AH1" s="39"/>
-      <c r="AI1" s="39"/>
-      <c r="AJ1" s="39"/>
-      <c r="AK1" s="39"/>
-      <c r="AL1" s="39"/>
-      <c r="AM1" s="39"/>
-      <c r="AN1" s="39"/>
-      <c r="AO1" s="39"/>
-      <c r="AP1" s="39"/>
-      <c r="AQ1" s="39"/>
-      <c r="AR1" s="39"/>
-      <c r="AS1" s="39"/>
-      <c r="AT1" s="39"/>
-      <c r="AU1" s="39"/>
-      <c r="AV1" s="39"/>
-      <c r="AW1" s="39"/>
-      <c r="AX1" s="39"/>
-      <c r="AY1" s="39"/>
-      <c r="AZ1" s="39"/>
-      <c r="BA1" s="39"/>
-      <c r="BB1" s="39"/>
-      <c r="BC1" s="39"/>
-      <c r="BD1" s="39"/>
-      <c r="BE1" s="39"/>
-      <c r="BF1" s="39"/>
-      <c r="BG1" s="39"/>
-      <c r="BH1" s="39"/>
-      <c r="BI1" s="39"/>
-      <c r="BJ1" s="39"/>
-      <c r="BK1" s="38" t="s">
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="33"/>
+      <c r="AH1" s="33"/>
+      <c r="AI1" s="33"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" s="38"/>
-      <c r="BM1" s="38"/>
-      <c r="BN1" s="34" t="s">
+      <c r="BL1" s="32"/>
+      <c r="BM1" s="32"/>
+      <c r="BN1" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" s="34"/>
-      <c r="BP1" s="34"/>
-      <c r="BQ1" s="34"/>
-    </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="BO1" s="28"/>
+      <c r="BP1" s="28"/>
+      <c r="BQ1" s="28"/>
+    </row>
+    <row r="2" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="14" t="s">
+      <c r="Q2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="R2" s="13" t="s">
         <v>167</v>
       </c>
       <c r="S2" s="4" t="s">
@@ -1962,22 +1948,22 @@
       <c r="AR2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AS2" s="18" t="s">
+      <c r="AS2" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AT2" s="18" t="s">
+      <c r="AT2" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AU2" s="18" t="s">
+      <c r="AU2" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AV2" s="18" t="s">
+      <c r="AV2" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="AW2" s="18" t="s">
+      <c r="AW2" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="AX2" s="18" t="s">
+      <c r="AX2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="AY2" s="7" t="s">
@@ -2016,30 +2002,30 @@
       <c r="BJ2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="BK2" s="10" t="s">
+      <c r="BK2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="BL2" s="10" t="s">
+      <c r="BL2" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="BM2" s="10" t="s">
+      <c r="BM2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="BN2" s="11" t="s">
+      <c r="BN2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="BO2" s="11" t="s">
+      <c r="BO2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="BP2" s="25" t="s">
+      <c r="BP2" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="BQ2" s="25" t="s">
+      <c r="BQ2" s="22" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -2054,16 +2040,16 @@
       <c r="E3">
         <v>112.439201</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G3" s="31">
+      <c r="G3" s="25">
         <v>0.37638888888888888</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I3" s="31">
+      <c r="I3" s="25">
         <v>0.42222222222222222</v>
       </c>
       <c r="J3">
@@ -2072,10 +2058,10 @@
       <c r="L3" t="s">
         <v>174</v>
       </c>
-      <c r="S3" s="30" t="s">
+      <c r="S3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T3" s="32">
+      <c r="T3" s="26">
         <v>0.82598379629629637</v>
       </c>
       <c r="U3">
@@ -2121,7 +2107,7 @@
         <v>7.2</v>
       </c>
       <c r="AU3">
-        <v>0.49299999999999999</v>
+        <v>493</v>
       </c>
       <c r="AV3">
         <v>8.58</v>
@@ -2138,15 +2124,15 @@
       <c r="BO3">
         <v>407.42</v>
       </c>
-      <c r="BP3" s="30">
+      <c r="BP3" s="24">
         <v>44417</v>
       </c>
-      <c r="BQ3" s="32">
+      <c r="BQ3" s="26">
         <v>0.90543981481481473</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -2161,16 +2147,16 @@
       <c r="E4">
         <v>112.43634900000001</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="25">
         <v>0.41319444444444442</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="H4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="25">
         <v>0.64583333333333337</v>
       </c>
       <c r="J4">
@@ -2182,10 +2168,10 @@
       <c r="M4" t="s">
         <v>210</v>
       </c>
-      <c r="S4" s="30" t="s">
+      <c r="S4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T4" s="32">
+      <c r="T4" s="26">
         <v>8.1851851851851856E-2</v>
       </c>
       <c r="U4">
@@ -2248,15 +2234,15 @@
       <c r="BO4">
         <v>409.18</v>
       </c>
-      <c r="BP4" s="30">
+      <c r="BP4" s="24">
         <v>44418</v>
       </c>
-      <c r="BQ4" s="32">
+      <c r="BQ4" s="26">
         <v>0.11388888888888889</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -2274,10 +2260,10 @@
       <c r="R5" t="s">
         <v>215</v>
       </c>
-      <c r="S5" s="30" t="s">
+      <c r="S5" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="T5" s="33">
+      <c r="T5" s="27">
         <v>1.2100578703703704</v>
       </c>
       <c r="U5">
@@ -2344,8 +2330,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -2360,16 +2346,16 @@
       <c r="E6">
         <v>112.447816</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="25">
         <v>0.48749999999999999</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="25">
         <v>0.51666666666666672</v>
       </c>
       <c r="J6">
@@ -2384,10 +2370,10 @@
       <c r="P6" t="s">
         <v>178</v>
       </c>
-      <c r="S6" s="30" t="s">
+      <c r="S6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="26">
         <v>0.93321759259259263</v>
       </c>
       <c r="U6">
@@ -2445,8 +2431,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -2461,16 +2447,16 @@
       <c r="E7">
         <v>112.450141</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="25">
         <v>0.50347222222222221</v>
       </c>
-      <c r="H7" s="30" t="s">
+      <c r="H7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="25">
         <v>0.52777777777777779</v>
       </c>
       <c r="J7">
@@ -2485,10 +2471,10 @@
       <c r="P7" t="s">
         <v>181</v>
       </c>
-      <c r="S7" s="30" t="s">
+      <c r="S7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T7" s="32">
+      <c r="T7" s="26">
         <v>0.92736111111111119</v>
       </c>
       <c r="U7">
@@ -2546,8 +2532,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -2565,10 +2551,10 @@
       <c r="R8" t="s">
         <v>216</v>
       </c>
-      <c r="S8" s="30" t="s">
+      <c r="S8" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T8" s="32">
+      <c r="T8" s="26">
         <v>0.94166666666666676</v>
       </c>
       <c r="U8">
@@ -2626,8 +2612,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A9" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B9" t="s">
@@ -2645,10 +2631,10 @@
       <c r="R9" t="s">
         <v>216</v>
       </c>
-      <c r="S9" s="30" t="s">
+      <c r="S9" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T9" s="32">
+      <c r="T9" s="26">
         <v>0.95173611111111101</v>
       </c>
       <c r="U9">
@@ -2706,8 +2692,8 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A10" s="24" t="s">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A10" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B10" t="s">
@@ -2722,16 +2708,16 @@
       <c r="E10">
         <v>112.44584399999999</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="25">
         <v>0.53472222222222221</v>
       </c>
-      <c r="H10" s="30" t="s">
+      <c r="H10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="25">
         <v>0.5541666666666667</v>
       </c>
       <c r="J10">
@@ -2740,10 +2726,10 @@
       <c r="L10" t="s">
         <v>182</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="S10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T10" s="32">
+      <c r="T10" s="26">
         <v>0.96045138888888892</v>
       </c>
       <c r="U10">
@@ -2801,8 +2787,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A11" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B11" t="s">
@@ -2817,16 +2803,16 @@
       <c r="E11">
         <v>112.441974</v>
       </c>
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G11" s="31">
+      <c r="G11" s="25">
         <v>0.54583333333333328</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="H11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="25">
         <v>0.56597222222222221</v>
       </c>
       <c r="J11">
@@ -2841,10 +2827,10 @@
       <c r="P11" t="s">
         <v>185</v>
       </c>
-      <c r="S11" s="30" t="s">
+      <c r="S11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T11" s="32">
+      <c r="T11" s="26">
         <v>0.97037037037037033</v>
       </c>
       <c r="U11">
@@ -2902,8 +2888,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A12" s="24" t="s">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A12" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B12" t="s">
@@ -2918,14 +2904,14 @@
       <c r="E12">
         <v>112.445359</v>
       </c>
-      <c r="F12" s="30"/>
+      <c r="F12" s="24"/>
       <c r="R12" t="s">
         <v>216</v>
       </c>
-      <c r="S12" s="30" t="s">
+      <c r="S12" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T12" s="32">
+      <c r="T12" s="26">
         <v>2.1006944444444443E-2</v>
       </c>
       <c r="U12">
@@ -2983,8 +2969,8 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
+    <row r="13" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A13" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B13" t="s">
@@ -2999,25 +2985,25 @@
       <c r="E13">
         <v>112.44264699999999</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="25">
         <v>0.56388888888888888</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="25">
         <v>0.57500000000000007</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
-      <c r="S13" s="30" t="s">
+      <c r="S13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T13" s="32">
+      <c r="T13" s="26">
         <v>0.97891203703703711</v>
       </c>
       <c r="U13">
@@ -3075,8 +3061,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
+    <row r="14" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A14" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B14" t="s">
@@ -3094,10 +3080,10 @@
       <c r="R14" t="s">
         <v>217</v>
       </c>
-      <c r="S14" s="30" t="s">
+      <c r="S14" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T14" s="32">
+      <c r="T14" s="26">
         <v>5.6134259259259271E-3</v>
       </c>
       <c r="U14">
@@ -3155,8 +3141,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A15" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B15" t="s">
@@ -3171,14 +3157,14 @@
       <c r="E15">
         <v>112.43522900000001</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="24"/>
       <c r="R15" t="s">
         <v>218</v>
       </c>
-      <c r="S15" s="30" t="s">
+      <c r="S15" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T15" s="32">
+      <c r="T15" s="26">
         <v>7.7314814814814822E-2</v>
       </c>
       <c r="U15">
@@ -3236,8 +3222,8 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A16" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B16" t="s">
@@ -3252,16 +3238,16 @@
       <c r="E16">
         <v>112.432439</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="25">
         <v>0.50138888888888888</v>
       </c>
-      <c r="H16" s="30" t="s">
+      <c r="H16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="25">
         <v>0.63194444444444442</v>
       </c>
       <c r="J16">
@@ -3270,10 +3256,10 @@
       <c r="K16" t="s">
         <v>211</v>
       </c>
-      <c r="S16" s="30" t="s">
+      <c r="S16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T16" s="32">
+      <c r="T16" s="26">
         <v>4.0972222222222222E-2</v>
       </c>
       <c r="U16">
@@ -3331,8 +3317,8 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+    <row r="17" spans="1:50" x14ac:dyDescent="0.5">
+      <c r="A17" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B17" t="s">
@@ -3347,16 +3333,16 @@
       <c r="E17">
         <v>112.4300246</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="25">
         <v>0.5083333333333333</v>
       </c>
-      <c r="H17" s="30" t="s">
+      <c r="H17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="25">
         <v>0.65625</v>
       </c>
       <c r="J17">
@@ -3365,10 +3351,10 @@
       <c r="K17" t="s">
         <v>211</v>
       </c>
-      <c r="S17" s="30" t="s">
+      <c r="S17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T17" s="32">
+      <c r="T17" s="26">
         <v>6.340277777777778E-2</v>
       </c>
       <c r="U17">
@@ -3444,727 +3430,726 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{229CFC7D-096F-4A49-B44F-3C66E059D51A}">
   <dimension ref="A1:C73"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.1171875" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" style="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="116.6640625" style="26" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="26"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.64453125" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A1" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:3" ht="71.7" x14ac:dyDescent="0.5">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="23" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="26" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A15" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="26" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A19" t="s">
         <v>166</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" t="s">
         <v>170</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="C19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A20" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A21" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="26" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" t="s">
         <v>138</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="26" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A24" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="26" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A25" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="26" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A26" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" t="s">
         <v>170</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A27" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A28" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="26" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A29" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="B29" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="C29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="26" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A31" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="26" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A32" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="26" t="s">
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="26" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A33" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="B33" t="s">
         <v>96</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="26" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A34" t="s">
         <v>148</v>
       </c>
-      <c r="B34" s="26" t="s">
+      <c r="B34" t="s">
         <v>97</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="26" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" t="s">
         <v>99</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="26" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A36" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="26" t="s">
+      <c r="B36" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="26" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="26" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="26" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="26" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="26" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="26" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="26" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="26" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A44" t="s">
         <v>140</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="B44" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="26" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A45" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="26" t="s">
+      <c r="B45" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="26" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A46" t="s">
         <v>150</v>
       </c>
-      <c r="B46" s="26" t="s">
+      <c r="B46" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A47" t="s">
         <v>142</v>
       </c>
-      <c r="B47" s="26" t="s">
+      <c r="B47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A48" t="s">
         <v>29</v>
       </c>
-      <c r="B48" s="26" t="s">
+      <c r="B48" t="s">
         <v>119</v>
       </c>
-      <c r="C48" s="26" t="s">
+      <c r="C48" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="26" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A49" t="s">
         <v>30</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B49" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="26" t="s">
+      <c r="C49" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="26" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
         <v>31</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B50" t="s">
         <v>108</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C50" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="26" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A51" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="26" t="s">
+      <c r="B51" t="s">
         <v>109</v>
       </c>
-      <c r="C51" s="26" t="s">
+      <c r="C51" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="26" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A52" t="s">
         <v>33</v>
       </c>
-      <c r="B52" s="26" t="s">
+      <c r="B52" t="s">
         <v>110</v>
       </c>
-      <c r="C52" s="26" t="s">
+      <c r="C52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="26" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
         <v>151</v>
       </c>
-      <c r="B53" s="26" t="s">
+      <c r="B53" t="s">
         <v>111</v>
       </c>
-      <c r="C53" s="26" t="s">
+      <c r="C53" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="26" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="26" t="s">
+      <c r="B54" t="s">
         <v>112</v>
       </c>
-      <c r="C54" s="26" t="s">
+      <c r="C54" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="26" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
         <v>40</v>
       </c>
-      <c r="B55" s="26" t="s">
+      <c r="B55" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="26" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A56" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="26" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="26" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="26" t="s">
+      <c r="B58" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="26" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
         <v>152</v>
       </c>
-      <c r="B59" s="26" t="s">
+      <c r="B59" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="26" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="26" t="s">
+      <c r="B60" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="26" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="26" t="s">
+      <c r="B61" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="26" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
         <v>144</v>
       </c>
-      <c r="B62" s="26" t="s">
+      <c r="B62" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="26" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
         <v>145</v>
       </c>
-      <c r="B63" s="26" t="s">
+      <c r="B63" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="26" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A64" t="s">
         <v>146</v>
       </c>
-      <c r="B64" s="26" t="s">
+      <c r="B64" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="26" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A65" t="s">
         <v>153</v>
       </c>
-      <c r="B65" s="26" t="s">
+      <c r="B65" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="26" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A66" t="s">
         <v>147</v>
       </c>
-      <c r="B66" s="26" t="s">
+      <c r="B66" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="26" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A67" t="s">
         <v>49</v>
       </c>
-      <c r="B67" s="26" t="s">
+      <c r="B67" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="26" t="s">
+      <c r="C67" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="26" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A68" t="s">
         <v>50</v>
       </c>
-      <c r="B68" s="26" t="s">
+      <c r="B68" t="s">
         <v>121</v>
       </c>
-      <c r="C68" s="26" t="s">
+      <c r="C68" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="26" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A69" t="s">
         <v>51</v>
       </c>
-      <c r="B69" s="26" t="s">
+      <c r="B69" t="s">
         <v>122</v>
       </c>
-      <c r="C69" s="26" t="s">
+      <c r="C69" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="26" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A70" t="s">
         <v>52</v>
       </c>
-      <c r="B70" s="26" t="s">
+      <c r="B70" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="26" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A71" t="s">
         <v>53</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" t="s">
         <v>161</v>
       </c>
-      <c r="C71" s="26" t="s">
+      <c r="C71" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="26" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A72" t="s">
         <v>162</v>
       </c>
-      <c r="B72" s="26" t="s">
+      <c r="B72" t="s">
         <v>163</v>
       </c>
-      <c r="C72" s="26" t="s">
+      <c r="C72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="26" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A73" t="s">
         <v>164</v>
       </c>
-      <c r="B73" s="26" t="s">
+      <c r="B73" t="s">
         <v>165</v>
       </c>
-      <c r="C73" s="26" t="s">
+      <c r="C73" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4176,33 +4161,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081A6BD0-DB1A-406D-A526-8D337C57DAFE}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="24"/>
-    <col min="3" max="3" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8.87890625" style="21"/>
+    <col min="3" max="3" width="15.41015625" customWidth="1"/>
+    <col min="5" max="5" width="13.3515625" customWidth="1"/>
+    <col min="7" max="7" width="12.3515625" customWidth="1"/>
+    <col min="9" max="9" width="14.3515625" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A1" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4218,7 +4200,7 @@
       <c r="E2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -4236,8 +4218,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -4265,8 +4247,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -4294,8 +4276,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -4323,8 +4305,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -4352,8 +4334,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -4381,8 +4363,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -4422,14 +4404,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FA2781-11F0-42BE-92DB-835D44D19C85}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5546875" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.52734375" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -4440,7 +4422,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4451,7 +4433,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -4462,19 +4444,19 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A4" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B5" t="s">
@@ -4484,8 +4466,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
@@ -4495,16 +4477,16 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" s="18" t="s">
         <v>123</v>
       </c>
       <c r="B8" t="s">
@@ -4514,8 +4496,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" s="18" t="s">
         <v>124</v>
       </c>
       <c r="B9" t="s">
@@ -4525,8 +4507,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" s="19" t="s">
         <v>125</v>
       </c>
       <c r="B10" t="s">
@@ -4536,8 +4518,8 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" s="18" t="s">
         <v>158</v>
       </c>
       <c r="B11" t="s">
@@ -4553,48 +4535,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5065,21 +5019,88 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="8b03727f-4454-4722-b3e6-018d8dcaf2fd"/>
+    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5091,24 +5112,4 @@
     <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Buoyancy frequency calculation fix, adding profile for lake 71, changed conductivity value in lake 71 datasheet
</commit_message>
<xml_diff>
--- a/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
+++ b/SuRGE_Sharepoint/data/CIN/CH4_071_Willowcreek/dataSheets/surgeData071.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/SuRGE/Shared Documents/data/CIN/CH4_071_Willowcreek/dataSheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\SuRGE\SuRGE_Sharepoint\data\CIN\CH4_071_Willowcreek\dataSheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="282" documentId="8_{C5CD2E9A-AC55-4F52-A58C-8568A1DAE714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C971E05-7B7B-4C6F-B545-53C2D1394674}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF5E157-2B73-4701-9FD2-A39D36E09D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13866" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -1225,7 +1225,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1247,9 +1247,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -1275,11 +1272,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1288,14 +1281,7 @@
     <xf numFmtId="49" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1380,9 +1366,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1420,7 +1406,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1526,7 +1512,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1668,7 +1654,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1677,211 +1663,211 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BQ17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" style="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.64453125" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.3515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.88671875" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.87890625" customWidth="1"/>
+    <col min="6" max="6" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.52734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.87890625" customWidth="1"/>
+    <col min="18" max="18" width="15.41015625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.64453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.87890625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.41015625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.64453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.87890625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="14.41015625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="6.87890625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.64453125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.44140625" customWidth="1"/>
-    <col min="30" max="30" width="6.109375" customWidth="1"/>
+    <col min="29" max="29" width="6.41015625" customWidth="1"/>
+    <col min="30" max="30" width="6.1171875" customWidth="1"/>
     <col min="31" max="31" width="6" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.64453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.52734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="12.87890625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.3515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.64453125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.3515625" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.64453125" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.41015625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.64453125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="14.87890625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="14.64453125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.3515625" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="8" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="6.44140625" customWidth="1"/>
-    <col min="49" max="49" width="5.6640625" customWidth="1"/>
-    <col min="50" max="50" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="6.41015625" customWidth="1"/>
+    <col min="49" max="49" width="5.64453125" customWidth="1"/>
+    <col min="50" max="50" width="6.3515625" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="11" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11.64453125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="13.3515625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.52734375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="8.87890625" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="10" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="16.1171875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="17.1171875" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="18.3515625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="13.64453125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="14" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="63" max="65" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="66" max="67" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="15.1171875" bestFit="1" customWidth="1"/>
+    <col min="63" max="65" width="9.1171875" bestFit="1" customWidth="1"/>
+    <col min="66" max="67" width="9.3515625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.41015625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.3515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A1" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="36" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="37" t="s">
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="39" t="s">
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" s="39"/>
-      <c r="Z1" s="39"/>
-      <c r="AA1" s="39"/>
-      <c r="AB1" s="39"/>
-      <c r="AC1" s="39"/>
-      <c r="AD1" s="39"/>
-      <c r="AE1" s="39"/>
-      <c r="AF1" s="39"/>
-      <c r="AG1" s="39"/>
-      <c r="AH1" s="39"/>
-      <c r="AI1" s="39"/>
-      <c r="AJ1" s="39"/>
-      <c r="AK1" s="39"/>
-      <c r="AL1" s="39"/>
-      <c r="AM1" s="39"/>
-      <c r="AN1" s="39"/>
-      <c r="AO1" s="39"/>
-      <c r="AP1" s="39"/>
-      <c r="AQ1" s="39"/>
-      <c r="AR1" s="39"/>
-      <c r="AS1" s="39"/>
-      <c r="AT1" s="39"/>
-      <c r="AU1" s="39"/>
-      <c r="AV1" s="39"/>
-      <c r="AW1" s="39"/>
-      <c r="AX1" s="39"/>
-      <c r="AY1" s="39"/>
-      <c r="AZ1" s="39"/>
-      <c r="BA1" s="39"/>
-      <c r="BB1" s="39"/>
-      <c r="BC1" s="39"/>
-      <c r="BD1" s="39"/>
-      <c r="BE1" s="39"/>
-      <c r="BF1" s="39"/>
-      <c r="BG1" s="39"/>
-      <c r="BH1" s="39"/>
-      <c r="BI1" s="39"/>
-      <c r="BJ1" s="39"/>
-      <c r="BK1" s="38" t="s">
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="33"/>
+      <c r="AH1" s="33"/>
+      <c r="AI1" s="33"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="BL1" s="38"/>
-      <c r="BM1" s="38"/>
-      <c r="BN1" s="34" t="s">
+      <c r="BL1" s="32"/>
+      <c r="BM1" s="32"/>
+      <c r="BN1" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="BO1" s="34"/>
-      <c r="BP1" s="34"/>
-      <c r="BQ1" s="34"/>
-    </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="BO1" s="28"/>
+      <c r="BP1" s="28"/>
+      <c r="BQ1" s="28"/>
+    </row>
+    <row r="2" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="14" t="s">
+      <c r="K2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="M2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="14" t="s">
+      <c r="Q2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="R2" s="13" t="s">
         <v>167</v>
       </c>
       <c r="S2" s="4" t="s">
@@ -1962,22 +1948,22 @@
       <c r="AR2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="AS2" s="18" t="s">
+      <c r="AS2" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="AT2" s="18" t="s">
+      <c r="AT2" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="AU2" s="18" t="s">
+      <c r="AU2" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="AV2" s="18" t="s">
+      <c r="AV2" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="AW2" s="18" t="s">
+      <c r="AW2" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="AX2" s="18" t="s">
+      <c r="AX2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="AY2" s="7" t="s">
@@ -2016,30 +2002,30 @@
       <c r="BJ2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="BK2" s="10" t="s">
+      <c r="BK2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="BL2" s="10" t="s">
+      <c r="BL2" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="BM2" s="10" t="s">
+      <c r="BM2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="BN2" s="11" t="s">
+      <c r="BN2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="BO2" s="11" t="s">
+      <c r="BO2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="BP2" s="25" t="s">
+      <c r="BP2" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="BQ2" s="25" t="s">
+      <c r="BQ2" s="22" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -2054,16 +2040,16 @@
       <c r="E3">
         <v>112.439201</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G3" s="31">
+      <c r="G3" s="25">
         <v>0.37638888888888888</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I3" s="31">
+      <c r="I3" s="25">
         <v>0.42222222222222222</v>
       </c>
       <c r="J3">
@@ -2072,10 +2058,10 @@
       <c r="L3" t="s">
         <v>174</v>
       </c>
-      <c r="S3" s="30" t="s">
+      <c r="S3" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T3" s="32">
+      <c r="T3" s="26">
         <v>0.82598379629629637</v>
       </c>
       <c r="U3">
@@ -2121,7 +2107,7 @@
         <v>7.2</v>
       </c>
       <c r="AU3">
-        <v>0.49299999999999999</v>
+        <v>493</v>
       </c>
       <c r="AV3">
         <v>8.58</v>
@@ -2138,15 +2124,15 @@
       <c r="BO3">
         <v>407.42</v>
       </c>
-      <c r="BP3" s="30">
+      <c r="BP3" s="24">
         <v>44417</v>
       </c>
-      <c r="BQ3" s="32">
+      <c r="BQ3" s="26">
         <v>0.90543981481481473</v>
       </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -2161,16 +2147,16 @@
       <c r="E4">
         <v>112.43634900000001</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="25">
         <v>0.41319444444444442</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="H4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="31">
+      <c r="I4" s="25">
         <v>0.64583333333333337</v>
       </c>
       <c r="J4">
@@ -2182,10 +2168,10 @@
       <c r="M4" t="s">
         <v>210</v>
       </c>
-      <c r="S4" s="30" t="s">
+      <c r="S4" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T4" s="32">
+      <c r="T4" s="26">
         <v>8.1851851851851856E-2</v>
       </c>
       <c r="U4">
@@ -2248,15 +2234,15 @@
       <c r="BO4">
         <v>409.18</v>
       </c>
-      <c r="BP4" s="30">
+      <c r="BP4" s="24">
         <v>44418</v>
       </c>
-      <c r="BQ4" s="32">
+      <c r="BQ4" s="26">
         <v>0.11388888888888889</v>
       </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -2274,10 +2260,10 @@
       <c r="R5" t="s">
         <v>215</v>
       </c>
-      <c r="S5" s="30" t="s">
+      <c r="S5" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="T5" s="33">
+      <c r="T5" s="27">
         <v>1.2100578703703704</v>
       </c>
       <c r="U5">
@@ -2344,8 +2330,8 @@
         <v>194</v>
       </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -2360,16 +2346,16 @@
       <c r="E6">
         <v>112.447816</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="25">
         <v>0.48749999999999999</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I6" s="31">
+      <c r="I6" s="25">
         <v>0.51666666666666672</v>
       </c>
       <c r="J6">
@@ -2384,10 +2370,10 @@
       <c r="P6" t="s">
         <v>178</v>
       </c>
-      <c r="S6" s="30" t="s">
+      <c r="S6" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T6" s="32">
+      <c r="T6" s="26">
         <v>0.93321759259259263</v>
       </c>
       <c r="U6">
@@ -2445,8 +2431,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -2461,16 +2447,16 @@
       <c r="E7">
         <v>112.450141</v>
       </c>
-      <c r="F7" s="30" t="s">
+      <c r="F7" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="25">
         <v>0.50347222222222221</v>
       </c>
-      <c r="H7" s="30" t="s">
+      <c r="H7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I7" s="31">
+      <c r="I7" s="25">
         <v>0.52777777777777779</v>
       </c>
       <c r="J7">
@@ -2485,10 +2471,10 @@
       <c r="P7" t="s">
         <v>181</v>
       </c>
-      <c r="S7" s="30" t="s">
+      <c r="S7" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T7" s="32">
+      <c r="T7" s="26">
         <v>0.92736111111111119</v>
       </c>
       <c r="U7">
@@ -2546,8 +2532,8 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -2565,10 +2551,10 @@
       <c r="R8" t="s">
         <v>216</v>
       </c>
-      <c r="S8" s="30" t="s">
+      <c r="S8" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T8" s="32">
+      <c r="T8" s="26">
         <v>0.94166666666666676</v>
       </c>
       <c r="U8">
@@ -2626,8 +2612,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
+    <row r="9" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A9" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B9" t="s">
@@ -2645,10 +2631,10 @@
       <c r="R9" t="s">
         <v>216</v>
       </c>
-      <c r="S9" s="30" t="s">
+      <c r="S9" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T9" s="32">
+      <c r="T9" s="26">
         <v>0.95173611111111101</v>
       </c>
       <c r="U9">
@@ -2706,8 +2692,8 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A10" s="24" t="s">
+    <row r="10" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A10" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B10" t="s">
@@ -2722,16 +2708,16 @@
       <c r="E10">
         <v>112.44584399999999</v>
       </c>
-      <c r="F10" s="30" t="s">
+      <c r="F10" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="25">
         <v>0.53472222222222221</v>
       </c>
-      <c r="H10" s="30" t="s">
+      <c r="H10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="25">
         <v>0.5541666666666667</v>
       </c>
       <c r="J10">
@@ -2740,10 +2726,10 @@
       <c r="L10" t="s">
         <v>182</v>
       </c>
-      <c r="S10" s="30" t="s">
+      <c r="S10" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T10" s="32">
+      <c r="T10" s="26">
         <v>0.96045138888888892</v>
       </c>
       <c r="U10">
@@ -2801,8 +2787,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+    <row r="11" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A11" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B11" t="s">
@@ -2817,16 +2803,16 @@
       <c r="E11">
         <v>112.441974</v>
       </c>
-      <c r="F11" s="30" t="s">
+      <c r="F11" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G11" s="31">
+      <c r="G11" s="25">
         <v>0.54583333333333328</v>
       </c>
-      <c r="H11" s="30" t="s">
+      <c r="H11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I11" s="31">
+      <c r="I11" s="25">
         <v>0.56597222222222221</v>
       </c>
       <c r="J11">
@@ -2841,10 +2827,10 @@
       <c r="P11" t="s">
         <v>185</v>
       </c>
-      <c r="S11" s="30" t="s">
+      <c r="S11" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T11" s="32">
+      <c r="T11" s="26">
         <v>0.97037037037037033</v>
       </c>
       <c r="U11">
@@ -2902,8 +2888,8 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A12" s="24" t="s">
+    <row r="12" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A12" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B12" t="s">
@@ -2918,14 +2904,14 @@
       <c r="E12">
         <v>112.445359</v>
       </c>
-      <c r="F12" s="30"/>
+      <c r="F12" s="24"/>
       <c r="R12" t="s">
         <v>216</v>
       </c>
-      <c r="S12" s="30" t="s">
+      <c r="S12" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T12" s="32">
+      <c r="T12" s="26">
         <v>2.1006944444444443E-2</v>
       </c>
       <c r="U12">
@@ -2983,8 +2969,8 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
+    <row r="13" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A13" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B13" t="s">
@@ -2999,25 +2985,25 @@
       <c r="E13">
         <v>112.44264699999999</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="25">
         <v>0.56388888888888888</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="25">
         <v>0.57500000000000007</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
-      <c r="S13" s="30" t="s">
+      <c r="S13" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T13" s="32">
+      <c r="T13" s="26">
         <v>0.97891203703703711</v>
       </c>
       <c r="U13">
@@ -3075,8 +3061,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
+    <row r="14" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A14" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B14" t="s">
@@ -3094,10 +3080,10 @@
       <c r="R14" t="s">
         <v>217</v>
       </c>
-      <c r="S14" s="30" t="s">
+      <c r="S14" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T14" s="32">
+      <c r="T14" s="26">
         <v>5.6134259259259271E-3</v>
       </c>
       <c r="U14">
@@ -3155,8 +3141,8 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
+    <row r="15" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A15" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B15" t="s">
@@ -3171,14 +3157,14 @@
       <c r="E15">
         <v>112.43522900000001</v>
       </c>
-      <c r="F15" s="30"/>
+      <c r="F15" s="24"/>
       <c r="R15" t="s">
         <v>218</v>
       </c>
-      <c r="S15" s="30" t="s">
+      <c r="S15" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T15" s="32">
+      <c r="T15" s="26">
         <v>7.7314814814814822E-2</v>
       </c>
       <c r="U15">
@@ -3236,8 +3222,8 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+    <row r="16" spans="1:69" x14ac:dyDescent="0.5">
+      <c r="A16" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B16" t="s">
@@ -3252,16 +3238,16 @@
       <c r="E16">
         <v>112.432439</v>
       </c>
-      <c r="F16" s="30" t="s">
+      <c r="F16" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="25">
         <v>0.50138888888888888</v>
       </c>
-      <c r="H16" s="30" t="s">
+      <c r="H16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="25">
         <v>0.63194444444444442</v>
       </c>
       <c r="J16">
@@ -3270,10 +3256,10 @@
       <c r="K16" t="s">
         <v>211</v>
       </c>
-      <c r="S16" s="30" t="s">
+      <c r="S16" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T16" s="32">
+      <c r="T16" s="26">
         <v>4.0972222222222222E-2</v>
       </c>
       <c r="U16">
@@ -3331,8 +3317,8 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="17" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+    <row r="17" spans="1:50" x14ac:dyDescent="0.5">
+      <c r="A17" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B17" t="s">
@@ -3347,16 +3333,16 @@
       <c r="E17">
         <v>112.4300246</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="31">
+      <c r="G17" s="25">
         <v>0.5083333333333333</v>
       </c>
-      <c r="H17" s="30" t="s">
+      <c r="H17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="25">
         <v>0.65625</v>
       </c>
       <c r="J17">
@@ -3365,10 +3351,10 @@
       <c r="K17" t="s">
         <v>211</v>
       </c>
-      <c r="S17" s="30" t="s">
+      <c r="S17" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="T17" s="32">
+      <c r="T17" s="26">
         <v>6.340277777777778E-2</v>
       </c>
       <c r="U17">
@@ -3444,727 +3430,726 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{229CFC7D-096F-4A49-B44F-3C66E059D51A}">
   <dimension ref="A1:C73"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.1171875" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" style="26" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="116.6640625" style="26" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="26"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="116.64453125" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A1" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:3" ht="71.7" x14ac:dyDescent="0.5">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="26" t="s">
+      <c r="C5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="C7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="26" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" t="s">
         <v>74</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="26" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="23" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="26" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="26" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A15" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="B16" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="26" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="B17" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="26" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A19" t="s">
         <v>166</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" t="s">
         <v>170</v>
       </c>
-      <c r="C19" s="26" t="s">
+      <c r="C19" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A20" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A21" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" t="s">
         <v>82</v>
       </c>
-      <c r="C21" s="26" t="s">
+      <c r="C21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="26" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="26" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" t="s">
         <v>138</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="26" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A24" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" t="s">
         <v>86</v>
       </c>
-      <c r="C24" s="26" t="s">
+      <c r="C24" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="26" t="s">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A25" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="26" t="s">
+      <c r="C25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="26" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A26" t="s">
         <v>168</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="B26" t="s">
         <v>170</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="26" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A27" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A28" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="B28" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="26" t="s">
+      <c r="C28" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="26" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A29" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="B29" t="s">
         <v>90</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="C29" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="26" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="26" t="s">
+      <c r="C30" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="26" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A31" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="C31" s="26" t="s">
+      <c r="C31" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="26" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A32" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="26" t="s">
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="26" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A33" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="B33" t="s">
         <v>96</v>
       </c>
-      <c r="C33" s="26" t="s">
+      <c r="C33" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="26" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A34" t="s">
         <v>148</v>
       </c>
-      <c r="B34" s="26" t="s">
+      <c r="B34" t="s">
         <v>97</v>
       </c>
-      <c r="C34" s="26" t="s">
+      <c r="C34" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="26" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A35" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" t="s">
         <v>99</v>
       </c>
-      <c r="C35" s="26" t="s">
+      <c r="C35" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="26" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A36" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="26" t="s">
+      <c r="B36" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="26" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="26" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="26" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="26" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
         <v>149</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="26" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
         <v>39</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="26" t="s">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="26" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="26" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A44" t="s">
         <v>140</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="B44" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="26" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A45" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="26" t="s">
+      <c r="B45" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="26" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A46" t="s">
         <v>150</v>
       </c>
-      <c r="B46" s="26" t="s">
+      <c r="B46" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A47" t="s">
         <v>142</v>
       </c>
-      <c r="B47" s="26" t="s">
+      <c r="B47" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A48" t="s">
         <v>29</v>
       </c>
-      <c r="B48" s="26" t="s">
+      <c r="B48" t="s">
         <v>119</v>
       </c>
-      <c r="C48" s="26" t="s">
+      <c r="C48" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="26" t="s">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A49" t="s">
         <v>30</v>
       </c>
-      <c r="B49" s="26" t="s">
+      <c r="B49" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="26" t="s">
+      <c r="C49" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="26" t="s">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
         <v>31</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="B50" t="s">
         <v>108</v>
       </c>
-      <c r="C50" s="26" t="s">
+      <c r="C50" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="26" t="s">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A51" t="s">
         <v>32</v>
       </c>
-      <c r="B51" s="26" t="s">
+      <c r="B51" t="s">
         <v>109</v>
       </c>
-      <c r="C51" s="26" t="s">
+      <c r="C51" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="26" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A52" t="s">
         <v>33</v>
       </c>
-      <c r="B52" s="26" t="s">
+      <c r="B52" t="s">
         <v>110</v>
       </c>
-      <c r="C52" s="26" t="s">
+      <c r="C52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="26" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
         <v>151</v>
       </c>
-      <c r="B53" s="26" t="s">
+      <c r="B53" t="s">
         <v>111</v>
       </c>
-      <c r="C53" s="26" t="s">
+      <c r="C53" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="26" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
         <v>34</v>
       </c>
-      <c r="B54" s="26" t="s">
+      <c r="B54" t="s">
         <v>112</v>
       </c>
-      <c r="C54" s="26" t="s">
+      <c r="C54" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="26" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
         <v>40</v>
       </c>
-      <c r="B55" s="26" t="s">
+      <c r="B55" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="26" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A56" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="26" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
         <v>42</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="26" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="26" t="s">
+      <c r="B58" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="26" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
         <v>152</v>
       </c>
-      <c r="B59" s="26" t="s">
+      <c r="B59" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="26" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
         <v>44</v>
       </c>
-      <c r="B60" s="26" t="s">
+      <c r="B60" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="26" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="26" t="s">
+      <c r="B61" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="26" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
         <v>144</v>
       </c>
-      <c r="B62" s="26" t="s">
+      <c r="B62" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="26" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
         <v>145</v>
       </c>
-      <c r="B63" s="26" t="s">
+      <c r="B63" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="26" t="s">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A64" t="s">
         <v>146</v>
       </c>
-      <c r="B64" s="26" t="s">
+      <c r="B64" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="26" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A65" t="s">
         <v>153</v>
       </c>
-      <c r="B65" s="26" t="s">
+      <c r="B65" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="26" t="s">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A66" t="s">
         <v>147</v>
       </c>
-      <c r="B66" s="26" t="s">
+      <c r="B66" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="26" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A67" t="s">
         <v>49</v>
       </c>
-      <c r="B67" s="26" t="s">
+      <c r="B67" t="s">
         <v>120</v>
       </c>
-      <c r="C67" s="26" t="s">
+      <c r="C67" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="26" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A68" t="s">
         <v>50</v>
       </c>
-      <c r="B68" s="26" t="s">
+      <c r="B68" t="s">
         <v>121</v>
       </c>
-      <c r="C68" s="26" t="s">
+      <c r="C68" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="26" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A69" t="s">
         <v>51</v>
       </c>
-      <c r="B69" s="26" t="s">
+      <c r="B69" t="s">
         <v>122</v>
       </c>
-      <c r="C69" s="26" t="s">
+      <c r="C69" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="26" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A70" t="s">
         <v>52</v>
       </c>
-      <c r="B70" s="26" t="s">
+      <c r="B70" t="s">
         <v>160</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="26" t="s">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A71" t="s">
         <v>53</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" t="s">
         <v>161</v>
       </c>
-      <c r="C71" s="26" t="s">
+      <c r="C71" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="26" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A72" t="s">
         <v>162</v>
       </c>
-      <c r="B72" s="26" t="s">
+      <c r="B72" t="s">
         <v>163</v>
       </c>
-      <c r="C72" s="26" t="s">
+      <c r="C72" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="26" t="s">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A73" t="s">
         <v>164</v>
       </c>
-      <c r="B73" s="26" t="s">
+      <c r="B73" t="s">
         <v>165</v>
       </c>
-      <c r="C73" s="26" t="s">
+      <c r="C73" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4176,33 +4161,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{081A6BD0-DB1A-406D-A526-8D337C57DAFE}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="24"/>
-    <col min="3" max="3" width="15.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8.87890625" style="21"/>
+    <col min="3" max="3" width="15.41015625" customWidth="1"/>
+    <col min="5" max="5" width="13.3515625" customWidth="1"/>
+    <col min="7" max="7" width="12.3515625" customWidth="1"/>
+    <col min="9" max="9" width="14.3515625" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="40" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A1" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4218,7 +4200,7 @@
       <c r="E2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -4236,8 +4218,8 @@
       <c r="K2" s="3"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A3" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B3" t="s">
@@ -4265,8 +4247,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A4" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B4" t="s">
@@ -4294,8 +4276,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B5" t="s">
@@ -4323,8 +4305,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A6" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B6" t="s">
@@ -4352,8 +4334,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A7" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B7" t="s">
@@ -4381,8 +4363,8 @@
         <v>19.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.5">
+      <c r="A8" s="21" t="s">
         <v>172</v>
       </c>
       <c r="B8" t="s">
@@ -4422,14 +4404,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44FA2781-11F0-42BE-92DB-835D44D19C85}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.5546875" customWidth="1"/>
-    <col min="3" max="3" width="49.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.64453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="63.52734375" customWidth="1"/>
+    <col min="3" max="3" width="49.52734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>135</v>
       </c>
@@ -4440,7 +4422,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4451,7 +4433,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -4462,19 +4444,19 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A4" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B5" t="s">
@@ -4484,8 +4466,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
@@ -4495,16 +4477,16 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" s="18" t="s">
         <v>123</v>
       </c>
       <c r="B8" t="s">
@@ -4514,8 +4496,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" s="18" t="s">
         <v>124</v>
       </c>
       <c r="B9" t="s">
@@ -4525,8 +4507,8 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" s="19" t="s">
         <v>125</v>
       </c>
       <c r="B10" t="s">
@@ -4536,8 +4518,8 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" s="18" t="s">
         <v>158</v>
       </c>
       <c r="B11" t="s">
@@ -4553,48 +4535,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001AF5FC5DD832BE4DBA6B24560DD3ADC0" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d40b3e6283001fb57e5088f84fb23d5e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="8b03727f-4454-4722-b3e6-018d8dcaf2fd" xmlns:ns6="ed970698-2d60-4bab-a048-d9be527522d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="aadbb8160917885bdc8cfb32badaafe9" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5065,21 +5019,88 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-21T13:32:44+00:00</Document_x0020_Creation_x0020_Date>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed970698-2d60-4bab-a048-d9be527522d9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="8b03727f-4454-4722-b3e6-018d8dcaf2fd"/>
+    <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D26D44A-9508-4707-B138-18882E5BA6FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5091,24 +5112,4 @@
     <ds:schemaRef ds:uri="ed970698-2d60-4bab-a048-d9be527522d9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADC939ED-97B3-43F4-B32D-176C8CDF450B}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{845EA28A-135D-4CD8-9991-40FEAFECD172}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F4A5FCF-4499-487A-89B0-E215184C11DF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>